<commit_message>
fix(template): anonymize all payroll example identities
</commit_message>
<xml_diff>
--- a/saudi_hr/public/templates/professional_payroll_import_template.xlsx
+++ b/saudi_hr/public/templates/professional_payroll_import_template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="دليل الاستخدام" sheetId="1" r:id="Rf3b3377b8d504e16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مسير الرواتب" sheetId="2" r:id="Rc61e23d425b34efd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مثال مكتمل" sheetId="3" r:id="R4a97a5a1a1674143"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="دليل الاستخدام" sheetId="1" r:id="Rd247a6e7e1254f4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مسير الرواتب" sheetId="2" r:id="R7ff80fbc05084dcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مثال مكتمل" sheetId="3" r:id="R225944449da5436b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -581,7 +581,7 @@
         <x:color rgb="FF147D64"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9F6F2"/>
         </x:patternFill>
       </x:fill>
@@ -592,7 +592,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -603,7 +603,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -614,7 +614,7 @@
         <x:color rgb="FF147D64"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9F6F2"/>
         </x:patternFill>
       </x:fill>
@@ -625,7 +625,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -636,7 +636,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -8907,10 +8907,10 @@
     </x:row>
     <x:row r="5" ht="23" customHeight="1">
       <x:c r="A5" s="119" t="str">
-        <x:v>1001</x:v>
+        <x:v>DEMO-001</x:v>
       </x:c>
       <x:c r="B5" s="105" t="str">
-        <x:v>أحمد محمد</x:v>
+        <x:v>موظف تجريبي ١</x:v>
       </x:c>
       <x:c r="C5" s="105" t="str">
         <x:v>الإدارة العامة</x:v>
@@ -8979,10 +8979,10 @@
         <x:v>6595</x:v>
       </x:c>
       <x:c r="X5" s="121" t="str">
-        <x:v>1012345678</x:v>
+        <x:v>DEMO-ID-001</x:v>
       </x:c>
       <x:c r="Y5" s="121" t="str">
-        <x:v>GOSI-1001</x:v>
+        <x:v>DEMO-GOSI-001</x:v>
       </x:c>
       <x:c r="Z5" s="109" t="str">
         <x:f>IF(COUNTA(A5:B5)=0,"",IF(OR(A5="",B5="",C5="",G5=""),"بيانات ناقصة",IF(COUNTIFS($A$5:$A$204,A5,$C$5:$C$204,C5)&gt;1,"صف مكرر","جاهز")))</x:f>
@@ -8991,10 +8991,10 @@
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
       <x:c r="A6" s="120" t="str">
-        <x:v>1002</x:v>
+        <x:v>DEMO-002</x:v>
       </x:c>
       <x:c r="B6" s="106" t="str">
-        <x:v>سارة عبدالله</x:v>
+        <x:v>موظف تجريبي ٢</x:v>
       </x:c>
       <x:c r="C6" s="106" t="str">
         <x:v>المبيعات</x:v>
@@ -9063,10 +9063,10 @@
         <x:v>7958</x:v>
       </x:c>
       <x:c r="X6" s="122" t="str">
-        <x:v>1023456789</x:v>
+        <x:v>DEMO-ID-002</x:v>
       </x:c>
       <x:c r="Y6" s="122" t="str">
-        <x:v>GOSI-1002</x:v>
+        <x:v>DEMO-GOSI-002</x:v>
       </x:c>
       <x:c r="Z6" s="110" t="str">
         <x:f>IF(COUNTA(A6:B6)=0,"",IF(OR(A6="",B6="",C6="",G6=""),"بيانات ناقصة",IF(COUNTIFS($A$5:$A$204,A6,$C$5:$C$204,C6)&gt;1,"صف مكرر","جاهز")))</x:f>
@@ -9075,10 +9075,10 @@
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
       <x:c r="A7" s="120" t="str">
-        <x:v>1003</x:v>
+        <x:v>DEMO-003</x:v>
       </x:c>
       <x:c r="B7" s="106" t="str">
-        <x:v>خالد علي</x:v>
+        <x:v>موظف تجريبي ٣</x:v>
       </x:c>
       <x:c r="C7" s="106" t="str">
         <x:v>التشغيل</x:v>
@@ -9147,10 +9147,10 @@
         <x:v>5775</x:v>
       </x:c>
       <x:c r="X7" s="122" t="str">
-        <x:v>1034567890</x:v>
+        <x:v>DEMO-ID-003</x:v>
       </x:c>
       <x:c r="Y7" s="122" t="str">
-        <x:v>GOSI-1003</x:v>
+        <x:v>DEMO-GOSI-003</x:v>
       </x:c>
       <x:c r="Z7" s="110" t="str">
         <x:f>IF(COUNTA(A7:B7)=0,"",IF(OR(A7="",B7="",C7="",G7=""),"بيانات ناقصة",IF(COUNTIFS($A$5:$A$204,A7,$C$5:$C$204,C7)&gt;1,"صف مكرر","جاهز")))</x:f>

</xml_diff>